<commit_message>
fix: handle streaming text output and transliteration completion wait
</commit_message>
<xml_diff>
--- a/IT23325814_Assignment 1 - Test cases.xlsx
+++ b/IT23325814_Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tharindu\Desktop\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F6DBD6-D538-4B40-8C7C-4FD3CA8EAB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5E035BA-3D42-4087-A307-BAF00532BB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="158">
   <si>
     <t>TC ID</t>
   </si>
@@ -292,211 +292,208 @@
     <t>ada vandesay hodata sellam kara.</t>
   </si>
   <si>
+    <t>අද වැන්ඩසේ හොදට සෙල්ලම් කරා.</t>
+  </si>
+  <si>
     <t>Neg_Fun_0029</t>
   </si>
   <si>
     <t>heta match eka thiyenne premadasa pittaniye.</t>
   </si>
   <si>
+    <t>හෙට match එක ප්‍රේමදාස පිට්ටනියේ.</t>
+  </si>
+  <si>
     <t>Neg_Fun_0030</t>
   </si>
   <si>
-    <t>doctor mata allergic thiyenawa.</t>
-  </si>
-  <si>
-    <t>doctor මට allergic තියෙනවා.</t>
+    <t>ape niwase thamai 1st place une.</t>
+  </si>
+  <si>
+    <t>අපේ නිවාසේ තමයි 1st place වුණේ.</t>
   </si>
   <si>
     <t>Neg_Fun_0031</t>
   </si>
   <si>
-    <t>dabulle yanawanam sigiriyeth yamuda?</t>
-  </si>
-  <si>
-    <t>දඹුල්ලේ යනවනම් සිගිරියේත් යමුද?</t>
+    <t>mama 5s wathawak sri pade giya.</t>
+  </si>
+  <si>
+    <t>මම 5ස් වතාවක් ශ්‍රී පාදේ ගියා.</t>
   </si>
   <si>
     <t>Neg_Fun_0032</t>
   </si>
   <si>
-    <t>bhathiya saha santhush lassanata sing karanwa.</t>
-  </si>
-  <si>
-    <t>භාතිය සහ සන්තුෂ් ලස්සනට සින්ග් කරනවා.</t>
+    <t>mata Rs. 3500 k poliyata denna puluwanda?</t>
+  </si>
+  <si>
+    <t>මට Rs. 3500ක් පොළියට දෙන්න පුලුවන්ද?</t>
   </si>
   <si>
     <t>Neg_Fun_0033</t>
   </si>
   <si>
-    <t>api inne 3rd year 2nd semester eke.</t>
-  </si>
-  <si>
-    <t>අපි ඉන්නේ 3rd year 2nd semester එකේ.</t>
+    <t>Mata USD 5000k masekin hoyaganna puluwan. Habai LKR walin nam echchr bh.</t>
+  </si>
+  <si>
+    <t>මට USD 5000k මාසෙකින් හොයාගන්න පුළුවන්. හැබැයි LKR වලින් නම් එච්චර බැහැ.</t>
   </si>
   <si>
     <t>Neg_Fun_0034</t>
   </si>
   <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>mama school eken out una gamanma campus ekata awe 2022 aurudde dan 3rd year 2nd semester ekath iwara wenna lagai.</t>
-  </si>
-  <si>
-    <t>මම school එකෙන් out උන ගමන්ම campus එකට ආවේ 2022 අවුරුද්දේ දැන් 3rd year 2nd semester එකත් ඉවර වෙන්න ළඟයි.</t>
+    <t>api uda maluwata yanakota 5.45PM unaa.</t>
+  </si>
+  <si>
+    <t>අපි උඩ මළුවට යනකොට 5.45PM වුණා.</t>
   </si>
   <si>
     <t>Neg_Fun_0035</t>
   </si>
   <si>
-    <t>mata  RS 1000k maru karala denna.</t>
-  </si>
-  <si>
-    <t>මට  RS 1000ක් මාරු කරලා දෙන්න.</t>
+    <t>concert eka 10.00 AM start karanwa.</t>
+  </si>
+  <si>
+    <t>Concert එක 10.00AM start කරනවා.</t>
   </si>
   <si>
     <t>Neg_Fun_0036</t>
   </si>
   <si>
-    <t>borathel mila $10k wadi wela.</t>
-  </si>
-  <si>
-    <t>බොරතෙල් මිල 10ක් වැඩි වෙලා.</t>
-  </si>
-  <si>
     <t>Neg_Fun_0037</t>
   </si>
   <si>
-    <t>concert eka 10.00 AM start karanwa.</t>
-  </si>
-  <si>
-    <t>concert එක 10.00 AM ස්ටාර්ට් කරනවා.</t>
+    <t>final exam may 11 sita june 05 dakwa pewathwe.</t>
+  </si>
+  <si>
+    <t>final exam මැයි 11 සිට ජූනි 05 දක්වා පැවත්වේ.</t>
   </si>
   <si>
     <t>Neg_Fun_0038</t>
   </si>
   <si>
-    <t>colombo sita kandy bala gaman karana dumriya 6.00 PM walata colombo walin pitath wenawa.</t>
-  </si>
-  <si>
-    <t>කොළඹ සිට කැන්ඩි බලා ගමන් කරන දුම්රිය 6.00 PM වලට කොළඹ වලින් පිටත් වෙනවා.</t>
+    <t>me sem eka may 27 iwara wenawa next sem eka july 15 patan gannawa.</t>
+  </si>
+  <si>
+    <t>මේ sem එක මැයි 27 ඉවර වෙනවා next sem එක july 15 පටන් ගන්නවා.</t>
   </si>
   <si>
     <t>Neg_Fun_0039</t>
   </si>
   <si>
-    <t>final exam may 11 sita june 05 dakwa pewathwe.</t>
-  </si>
-  <si>
-    <t>final exam මැයි 11 සිට ජූනි 05 දක්වා පැවත්වේ.</t>
+    <t>victoria dem  eke usa feet 200ta wadi.</t>
+  </si>
+  <si>
+    <t>වික්ටෝරියා ඩෑම්  එකේ උස ෆීට් 200ට වැඩි.</t>
   </si>
   <si>
     <t>Neg_Fun_0040</t>
   </si>
   <si>
-    <t>me sem eka may 27 iwara wenawa next sem eka july 15 patan gannawa.</t>
-  </si>
-  <si>
-    <t>මේ sem එක මැයි 27 ඉවර වෙනවා next sem එක july 15 පටන් ගන්නවා.</t>
+    <t>fitness test eka pass wenna 5km 7 minutes walin duwanna wenawa.</t>
+  </si>
+  <si>
+    <t>fitness test එක pass වෙන්න 5km 7 minutes වලින් දුවන්න වෙනවා.</t>
   </si>
   <si>
     <t>Neg_Fun_0041</t>
   </si>
   <si>
-    <t>victoria dem  eke usa feet 200ta wadi.</t>
-  </si>
-  <si>
-    <t>වික්ටෝරියා ඩෑම්  එකේ උස ෆීට් 200ට වැඩි.</t>
+    <t>ado eka mara film ekak niyameta set una.</t>
   </si>
   <si>
     <t>Neg_Fun_0042</t>
   </si>
   <si>
-    <t>fitness test eka pass wenna 5km 7 minutes walin duwanna wenawa.</t>
-  </si>
-  <si>
-    <t>fitness test එක pass වෙන්න 5km 7 minutes වලින් දුවන්න වෙනවා.</t>
+    <t>ado uba hodata wede karala.</t>
   </si>
   <si>
     <t>Neg_Fun_0043</t>
   </si>
   <si>
-    <t>ado eka mara film ekak niyameta set una.</t>
-  </si>
-  <si>
-    <t>අඩො එක මාර ෆිල්ම් එකක් නියමෙට set උනා.</t>
+    <t>aluthma news balanna www.newsfirst.lk web ekata yanna.</t>
+  </si>
+  <si>
+    <t>අලුත්ම news බලන්න www.newsfirst.lk වෙබ් එකට යන්න.</t>
   </si>
   <si>
     <t>Neg_Fun_0044</t>
   </si>
   <si>
-    <t>ado uba hodata wede karala.</t>
-  </si>
-  <si>
-    <t>අඩො උඹ හොදට වැඩේ කරල.</t>
+    <t xml:space="preserve"> @everyone heta annual party eka.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> @everyone හෙට annual party එක.C186</t>
   </si>
   <si>
     <t>Neg_Fun_0045</t>
   </si>
   <si>
-    <t>aluthma news balanna www.newsfirst.lk web ekata yanna.</t>
-  </si>
-  <si>
-    <t>අලුත්ම news බලන්න www.newsfirst.lk වෙබ් එකට යන්න.</t>
+    <t>mata hinawa 😂 nawaththaganna bari una.</t>
   </si>
   <si>
     <t>Neg_Fun_0046</t>
   </si>
   <si>
-    <t xml:space="preserve"> @everyone heta annual party eka.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> @everyone හෙට annual party එක.C186</t>
+    <t>ado eka aul ban mata 😕.</t>
+  </si>
+  <si>
+    <t>අඩො ඒක අවුල් බන් මට 😕.</t>
   </si>
   <si>
     <t>Neg_Fun_0047</t>
   </si>
   <si>
-    <t>mata hinawa 😂 nawaththaganna bari una.</t>
-  </si>
-  <si>
-    <t>මට හිනාව 😂 නවත්තගන්න බැරි උනා.</t>
+    <t>bro mata kanagatui 😥.</t>
+  </si>
+  <si>
+    <t>bro මට කනගාටුයි 😥.</t>
   </si>
   <si>
     <t>Neg_Fun_0048</t>
   </si>
   <si>
-    <t>ado eka aul ban mata 😕.</t>
-  </si>
-  <si>
-    <t>අඩො ඒක අවුල් බන් මට 😕.</t>
+    <t>bro me semester eke marks hodata thibboth gpa eka hadaganna puluwan.</t>
   </si>
   <si>
     <t>Neg_Fun_0049</t>
   </si>
   <si>
-    <t>bro mata kanagatui 😥.</t>
-  </si>
-  <si>
-    <t>bro මට කනගාටුයි 😥.</t>
+    <t>uu nam maha buruwk 🤣</t>
+  </si>
+  <si>
+    <t>ඌ නම් මහා බූරුවෙක් 🤣</t>
   </si>
   <si>
     <t>Neg_Fun_0050</t>
   </si>
   <si>
-    <t>bro me semester eke marks hodata thibboth gpa eka hadaganna puluwan.</t>
-  </si>
-  <si>
-    <t>bro මේ semester එකේ marks හොදට තිබ්බොත් gpa එක හදාගන්න පුලුවන්.</t>
-  </si>
-  <si>
-    <t>අද වැන්ඩසේ හොදට සෙල්ලම් කරා.</t>
-  </si>
-  <si>
-    <t>හෙට match එක ප්‍රේමදාස පිට්ටනියේ.</t>
-  </si>
-  <si>
-    <t>oyaa adha lassanai. like a princess.</t>
+    <t>mata nam dan mala panala inne 😡</t>
+  </si>
+  <si>
+    <t>මට නම් දැන් මල පැනලා ඉන්නේ 😡</t>
+  </si>
+  <si>
+    <t>borathel mila ganan $10k wadi wela.</t>
+  </si>
+  <si>
+    <t>bro මේ semester එකේ marks හොදට තිබ්බොත් gpa එක හදාගන්න පුළුවන්.</t>
+  </si>
+  <si>
+    <t>මට හිනාව 😂 නවත්තගන්න බැරි වුණා.</t>
+  </si>
+  <si>
+    <t>අඩෝ උබ හොඳට වැඩේ කරලා.</t>
+  </si>
+  <si>
+    <t>අඩො එක මාර ෆිල්ම් එකක් නියමෙට set වුණා.</t>
+  </si>
+  <si>
+    <t>බොරතෙල් මිල ගණන් $10ක් වැඩි වෙලා.</t>
+  </si>
+  <si>
+    <t>oyaa adha lassanai. like a princes.</t>
   </si>
 </sst>
 </file>
@@ -596,7 +593,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -606,10 +603,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -618,10 +618,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -937,7 +933,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -946,11 +942,11 @@
       <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
     </row>
     <row r="3" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
@@ -977,7 +973,7 @@
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -986,11 +982,11 @@
       <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
@@ -1017,7 +1013,7 @@
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1026,11 +1022,11 @@
       <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="9"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
@@ -1057,7 +1053,7 @@
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -1066,11 +1062,11 @@
       <c r="C14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
     </row>
     <row r="15" spans="1:6" ht="1.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
@@ -1097,7 +1093,7 @@
       <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -1106,11 +1102,11 @@
       <c r="C18" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" ht="1.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
@@ -1137,7 +1133,7 @@
       <c r="F21" s="4"/>
     </row>
     <row r="22" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B22" s="2" t="s">
@@ -1146,11 +1142,11 @@
       <c r="C22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="7"/>
-      <c r="F22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
@@ -1177,7 +1173,7 @@
       <c r="F25" s="4"/>
     </row>
     <row r="26" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
@@ -1186,11 +1182,11 @@
       <c r="C26" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="9"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="6"/>
     </row>
     <row r="27" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
@@ -1217,7 +1213,7 @@
       <c r="F29" s="4"/>
     </row>
     <row r="30" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="7" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
@@ -1226,11 +1222,11 @@
       <c r="C30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3"/>
@@ -1257,7 +1253,7 @@
       <c r="F33" s="4"/>
     </row>
     <row r="34" spans="1:6" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B34" s="2" t="s">
@@ -1266,11 +1262,11 @@
       <c r="C34" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3"/>
@@ -1297,7 +1293,7 @@
       <c r="F37" s="4"/>
     </row>
     <row r="38" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B38" s="2" t="s">
@@ -1306,11 +1302,11 @@
       <c r="C38" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E38" s="7"/>
-      <c r="F38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="9"/>
     </row>
     <row r="39" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
@@ -1337,7 +1333,7 @@
       <c r="F41" s="4"/>
     </row>
     <row r="42" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="5" t="s">
         <v>38</v>
       </c>
       <c r="B42" s="2" t="s">
@@ -1346,11 +1342,11 @@
       <c r="C42" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="D42" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E42" s="7"/>
-      <c r="F42" s="9"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="6"/>
     </row>
     <row r="43" spans="1:6" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3"/>
@@ -1377,7 +1373,7 @@
       <c r="F45" s="4"/>
     </row>
     <row r="46" spans="1:6" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B46" s="2" t="s">
@@ -1386,11 +1382,11 @@
       <c r="C46" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="D46" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
     </row>
     <row r="47" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3"/>
@@ -1417,7 +1413,7 @@
       <c r="F49" s="4"/>
     </row>
     <row r="50" spans="1:6" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B50" s="2" t="s">
@@ -1426,11 +1422,11 @@
       <c r="C50" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="D50" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
     </row>
     <row r="51" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3"/>
@@ -1457,7 +1453,7 @@
       <c r="F53" s="4"/>
     </row>
     <row r="54" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="5" t="s">
         <v>47</v>
       </c>
       <c r="B54" s="2" t="s">
@@ -1466,11 +1462,11 @@
       <c r="C54" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="D54" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E54" s="7"/>
-      <c r="F54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="9"/>
     </row>
     <row r="55" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="3"/>
@@ -1497,20 +1493,20 @@
       <c r="F57" s="4"/>
     </row>
     <row r="58" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="D58" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="D58" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E58" s="7"/>
-      <c r="F58" s="9"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="6"/>
     </row>
     <row r="59" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="3"/>
@@ -1537,7 +1533,7 @@
       <c r="F61" s="4"/>
     </row>
     <row r="62" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="5" t="s">
+      <c r="A62" s="7" t="s">
         <v>52</v>
       </c>
       <c r="B62" s="2" t="s">
@@ -1546,11 +1542,11 @@
       <c r="C62" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="D62" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
     </row>
     <row r="63" spans="1:6" ht="0.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="3"/>
@@ -1577,7 +1573,7 @@
       <c r="F65" s="4"/>
     </row>
     <row r="66" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="6" t="s">
+      <c r="A66" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B66" s="2" t="s">
@@ -1586,11 +1582,11 @@
       <c r="C66" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E66" s="7"/>
-      <c r="F66" s="7"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="8"/>
     </row>
     <row r="67" spans="1:6" ht="1.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="3"/>
@@ -1617,7 +1613,7 @@
       <c r="F69" s="4"/>
     </row>
     <row r="70" spans="1:6" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="6" t="s">
+      <c r="A70" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B70" s="2" t="s">
@@ -1626,11 +1622,11 @@
       <c r="C70" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D70" s="5" t="s">
+      <c r="D70" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E70" s="7"/>
-      <c r="F70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="9"/>
     </row>
     <row r="71" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="3"/>
@@ -1657,7 +1653,7 @@
       <c r="F73" s="4"/>
     </row>
     <row r="74" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="6" t="s">
+      <c r="A74" s="5" t="s">
         <v>61</v>
       </c>
       <c r="B74" s="2" t="s">
@@ -1666,11 +1662,11 @@
       <c r="C74" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D74" s="5" t="s">
+      <c r="D74" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E74" s="7"/>
-      <c r="F74" s="9"/>
+      <c r="E74" s="8"/>
+      <c r="F74" s="6"/>
     </row>
     <row r="75" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="3"/>
@@ -1697,7 +1693,7 @@
       <c r="F77" s="4"/>
     </row>
     <row r="78" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="5" t="s">
+      <c r="A78" s="7" t="s">
         <v>64</v>
       </c>
       <c r="B78" s="2" t="s">
@@ -1706,11 +1702,11 @@
       <c r="C78" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
+      <c r="E78" s="7"/>
+      <c r="F78" s="7"/>
     </row>
     <row r="79" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="3"/>
@@ -1737,7 +1733,7 @@
       <c r="F81" s="4"/>
     </row>
     <row r="82" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="6" t="s">
+      <c r="A82" s="5" t="s">
         <v>67</v>
       </c>
       <c r="B82" s="2" t="s">
@@ -1746,11 +1742,11 @@
       <c r="C82" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D82" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E82" s="7"/>
-      <c r="F82" s="7"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
     </row>
     <row r="83" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="3"/>
@@ -1777,7 +1773,7 @@
       <c r="F85" s="4"/>
     </row>
     <row r="86" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="6" t="s">
+      <c r="A86" s="5" t="s">
         <v>70</v>
       </c>
       <c r="B86" s="2" t="s">
@@ -1786,11 +1782,11 @@
       <c r="C86" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D86" s="5" t="s">
+      <c r="D86" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E86" s="7"/>
-      <c r="F86" s="8"/>
+      <c r="E86" s="8"/>
+      <c r="F86" s="9"/>
     </row>
     <row r="87" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="3"/>
@@ -1817,7 +1813,7 @@
       <c r="F89" s="4"/>
     </row>
     <row r="90" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="6" t="s">
+      <c r="A90" s="5" t="s">
         <v>73</v>
       </c>
       <c r="B90" s="2" t="s">
@@ -1826,11 +1822,11 @@
       <c r="C90" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D90" s="5" t="s">
+      <c r="D90" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E90" s="7"/>
-      <c r="F90" s="9"/>
+      <c r="E90" s="8"/>
+      <c r="F90" s="6"/>
     </row>
     <row r="91" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="3"/>
@@ -1857,7 +1853,7 @@
       <c r="F93" s="4"/>
     </row>
     <row r="94" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="5" t="s">
+      <c r="A94" s="7" t="s">
         <v>76</v>
       </c>
       <c r="B94" s="2" t="s">
@@ -1866,11 +1862,11 @@
       <c r="C94" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D94" s="5" t="s">
+      <c r="D94" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E94" s="5"/>
-      <c r="F94" s="5"/>
+      <c r="E94" s="7"/>
+      <c r="F94" s="7"/>
     </row>
     <row r="95" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="3"/>
@@ -1897,7 +1893,7 @@
       <c r="F97" s="4"/>
     </row>
     <row r="98" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="6" t="s">
+      <c r="A98" s="5" t="s">
         <v>79</v>
       </c>
       <c r="B98" s="2" t="s">
@@ -1906,11 +1902,11 @@
       <c r="C98" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D98" s="5" t="s">
+      <c r="D98" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E98" s="7"/>
-      <c r="F98" s="7"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8"/>
     </row>
     <row r="99" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="3"/>
@@ -1937,7 +1933,7 @@
       <c r="F101" s="4"/>
     </row>
     <row r="102" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="6" t="s">
+      <c r="A102" s="5" t="s">
         <v>82</v>
       </c>
       <c r="B102" s="2" t="s">
@@ -1946,11 +1942,11 @@
       <c r="C102" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D102" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="E102" s="7"/>
-      <c r="F102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="9"/>
     </row>
     <row r="103" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="3"/>
@@ -1977,7 +1973,7 @@
       <c r="F105" s="4"/>
     </row>
     <row r="106" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="6" t="s">
+      <c r="A106" s="5" t="s">
         <v>85</v>
       </c>
       <c r="B106" s="2" t="s">
@@ -1986,11 +1982,11 @@
       <c r="C106" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D106" s="5" t="s">
+      <c r="D106" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E106" s="7"/>
-      <c r="F106" s="9"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="6"/>
     </row>
     <row r="107" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="3"/>
@@ -2017,7 +2013,7 @@
       <c r="F109" s="4"/>
     </row>
     <row r="110" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="5" t="s">
+      <c r="A110" s="7" t="s">
         <v>88</v>
       </c>
       <c r="B110" s="2" t="s">
@@ -2026,11 +2022,11 @@
       <c r="C110" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D110" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="E110" s="5"/>
-      <c r="F110" s="5"/>
+      <c r="D110" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E110" s="7"/>
+      <c r="F110" s="7"/>
     </row>
     <row r="111" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="3"/>
@@ -2057,20 +2053,20 @@
       <c r="F113" s="4"/>
     </row>
     <row r="114" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="6" t="s">
-        <v>90</v>
+      <c r="A114" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D114" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="E114" s="7"/>
-      <c r="F114" s="7"/>
+        <v>92</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E114" s="8"/>
+      <c r="F114" s="8"/>
     </row>
     <row r="115" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="3"/>
@@ -2097,20 +2093,20 @@
       <c r="F117" s="4"/>
     </row>
     <row r="118" spans="1:6" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="6" t="s">
-        <v>92</v>
+      <c r="A118" s="5" t="s">
+        <v>94</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="E118" s="7"/>
-      <c r="F118" s="8"/>
+        <v>95</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E118" s="8"/>
+      <c r="F118" s="9"/>
     </row>
     <row r="119" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="3"/>
@@ -2137,20 +2133,20 @@
       <c r="F121" s="4"/>
     </row>
     <row r="122" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="6" t="s">
-        <v>95</v>
+      <c r="A122" s="5" t="s">
+        <v>97</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D122" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="E122" s="7"/>
-      <c r="F122" s="9"/>
+        <v>98</v>
+      </c>
+      <c r="D122" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E122" s="8"/>
+      <c r="F122" s="6"/>
     </row>
     <row r="123" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="3"/>
@@ -2177,20 +2173,20 @@
       <c r="F125" s="4"/>
     </row>
     <row r="126" spans="1:6" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="5" t="s">
-        <v>98</v>
+      <c r="A126" s="7" t="s">
+        <v>100</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D126" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="E126" s="5"/>
-      <c r="F126" s="5"/>
+        <v>101</v>
+      </c>
+      <c r="D126" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E126" s="7"/>
+      <c r="F126" s="7"/>
     </row>
     <row r="127" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="3"/>
@@ -2217,20 +2213,20 @@
       <c r="F129" s="4"/>
     </row>
     <row r="130" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="6" t="s">
-        <v>101</v>
+      <c r="A130" s="5" t="s">
+        <v>103</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E130" s="7"/>
-      <c r="F130" s="7"/>
+        <v>104</v>
+      </c>
+      <c r="D130" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E130" s="8"/>
+      <c r="F130" s="8"/>
     </row>
     <row r="131" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="3"/>
@@ -2257,20 +2253,20 @@
       <c r="F133" s="4"/>
     </row>
     <row r="134" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="6" t="s">
-        <v>104</v>
+      <c r="A134" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>105</v>
+        <v>7</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D134" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E134" s="7"/>
-      <c r="F134" s="8"/>
+      <c r="D134" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E134" s="8"/>
+      <c r="F134" s="9"/>
     </row>
     <row r="135" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="3"/>
@@ -2297,20 +2293,20 @@
       <c r="F137" s="4"/>
     </row>
     <row r="138" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="6" t="s">
-        <v>108</v>
+      <c r="A138" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D138" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E138" s="7"/>
-      <c r="F138" s="9"/>
+      <c r="D138" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E138" s="8"/>
+      <c r="F138" s="6"/>
     </row>
     <row r="139" spans="1:6" ht="1.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="3"/>
@@ -2337,20 +2333,20 @@
       <c r="F141" s="4"/>
     </row>
     <row r="142" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="5" t="s">
-        <v>111</v>
+      <c r="A142" s="7" t="s">
+        <v>112</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D142" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="E142" s="5"/>
-      <c r="F142" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="D142" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="E142" s="7"/>
+      <c r="F142" s="7"/>
     </row>
     <row r="143" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="3"/>
@@ -2377,20 +2373,20 @@
       <c r="F145" s="4"/>
     </row>
     <row r="146" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="6" t="s">
+      <c r="A146" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C146" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B146" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C146" s="2" t="s">
+      <c r="D146" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D146" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="E146" s="7"/>
-      <c r="F146" s="7"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
     </row>
     <row r="147" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="3"/>
@@ -2417,20 +2413,20 @@
       <c r="F149" s="4"/>
     </row>
     <row r="150" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="6" t="s">
-        <v>117</v>
+      <c r="A150" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C150" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D150" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="D150" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="E150" s="7"/>
-      <c r="F150" s="8"/>
+      <c r="E150" s="8"/>
+      <c r="F150" s="9"/>
     </row>
     <row r="151" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="3"/>
@@ -2457,20 +2453,20 @@
       <c r="F153" s="4"/>
     </row>
     <row r="154" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="6" t="s">
-        <v>120</v>
+      <c r="A154" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="B154" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C154" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D154" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D154" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="E154" s="7"/>
-      <c r="F154" s="9"/>
+      <c r="E154" s="8"/>
+      <c r="F154" s="6"/>
     </row>
     <row r="155" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="3"/>
@@ -2497,20 +2493,20 @@
       <c r="F157" s="4"/>
     </row>
     <row r="158" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A158" s="5" t="s">
-        <v>123</v>
+      <c r="A158" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C158" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D158" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="D158" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="E158" s="5"/>
-      <c r="F158" s="5"/>
+      <c r="E158" s="7"/>
+      <c r="F158" s="7"/>
     </row>
     <row r="159" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="3"/>
@@ -2537,20 +2533,20 @@
       <c r="F161" s="4"/>
     </row>
     <row r="162" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="6" t="s">
-        <v>126</v>
+      <c r="A162" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D162" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E162" s="7"/>
-      <c r="F162" s="7"/>
+        <v>126</v>
+      </c>
+      <c r="D162" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="E162" s="8"/>
+      <c r="F162" s="8"/>
     </row>
     <row r="163" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="3"/>
@@ -2577,20 +2573,20 @@
       <c r="F165" s="4"/>
     </row>
     <row r="166" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="6" t="s">
-        <v>129</v>
+      <c r="A166" s="5" t="s">
+        <v>127</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="D166" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="E166" s="7"/>
-      <c r="F166" s="8"/>
+        <v>128</v>
+      </c>
+      <c r="D166" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="E166" s="8"/>
+      <c r="F166" s="9"/>
     </row>
     <row r="167" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="3"/>
@@ -2617,20 +2613,20 @@
       <c r="F169" s="4"/>
     </row>
     <row r="170" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="6" t="s">
-        <v>132</v>
+      <c r="A170" s="5" t="s">
+        <v>129</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D170" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="E170" s="7"/>
-      <c r="F170" s="9"/>
+        <v>130</v>
+      </c>
+      <c r="D170" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E170" s="8"/>
+      <c r="F170" s="6"/>
     </row>
     <row r="171" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="3"/>
@@ -2657,20 +2653,20 @@
       <c r="F173" s="4"/>
     </row>
     <row r="174" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="5" t="s">
-        <v>135</v>
+      <c r="A174" s="7" t="s">
+        <v>132</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D174" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E174" s="5"/>
-      <c r="F174" s="5"/>
+        <v>133</v>
+      </c>
+      <c r="D174" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E174" s="7"/>
+      <c r="F174" s="7"/>
     </row>
     <row r="175" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="3"/>
@@ -2697,20 +2693,20 @@
       <c r="F177" s="4"/>
     </row>
     <row r="178" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A178" s="6" t="s">
-        <v>138</v>
+      <c r="A178" s="5" t="s">
+        <v>135</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D178" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="E178" s="7"/>
-      <c r="F178" s="7"/>
+        <v>136</v>
+      </c>
+      <c r="D178" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E178" s="8"/>
+      <c r="F178" s="8"/>
     </row>
     <row r="179" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="3"/>
@@ -2737,20 +2733,20 @@
       <c r="F181" s="4"/>
     </row>
     <row r="182" spans="1:6" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A182" s="6" t="s">
-        <v>141</v>
+      <c r="A182" s="5" t="s">
+        <v>137</v>
       </c>
       <c r="B182" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D182" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E182" s="7"/>
-      <c r="F182" s="8"/>
+        <v>138</v>
+      </c>
+      <c r="D182" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E182" s="8"/>
+      <c r="F182" s="9"/>
     </row>
     <row r="183" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="3"/>
@@ -2777,20 +2773,20 @@
       <c r="F185" s="4"/>
     </row>
     <row r="186" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A186" s="6" t="s">
-        <v>144</v>
+      <c r="A186" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D186" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="E186" s="7"/>
-      <c r="F186" s="9"/>
+        <v>141</v>
+      </c>
+      <c r="D186" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E186" s="8"/>
+      <c r="F186" s="6"/>
     </row>
     <row r="187" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="3"/>
@@ -2817,20 +2813,20 @@
       <c r="F189" s="4"/>
     </row>
     <row r="190" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="5" t="s">
-        <v>147</v>
+      <c r="A190" s="7" t="s">
+        <v>143</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D190" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="E190" s="5"/>
-      <c r="F190" s="5"/>
+        <v>144</v>
+      </c>
+      <c r="D190" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E190" s="7"/>
+      <c r="F190" s="7"/>
     </row>
     <row r="191" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="3"/>
@@ -2857,20 +2853,20 @@
       <c r="F193" s="4"/>
     </row>
     <row r="194" spans="1:6" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A194" s="6" t="s">
-        <v>150</v>
+      <c r="A194" s="5" t="s">
+        <v>145</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="D194" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="E194" s="7"/>
-      <c r="F194" s="9"/>
+        <v>146</v>
+      </c>
+      <c r="D194" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="E194" s="8"/>
+      <c r="F194" s="6"/>
     </row>
     <row r="195" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="3"/>
@@ -2896,48 +2892,324 @@
       <c r="E197" s="4"/>
       <c r="F197" s="4"/>
     </row>
-    <row r="198" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A198" s="5" t="s">
-        <v>153</v>
+    <row r="198" spans="1:6" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A198" s="7" t="s">
+        <v>148</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="D198" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="E198" s="5"/>
-      <c r="F198" s="5"/>
+        <v>149</v>
+      </c>
+      <c r="D198" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E198" s="7"/>
+      <c r="F198" s="7"/>
     </row>
     <row r="199" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A199" s="10"/>
-      <c r="B199" s="10"/>
-      <c r="C199" s="10"/>
-      <c r="D199" s="10"/>
-      <c r="E199" s="10"/>
-      <c r="F199" s="10"/>
+      <c r="A199" s="3"/>
+      <c r="B199" s="3"/>
+      <c r="C199" s="3"/>
+      <c r="D199" s="3"/>
+      <c r="E199" s="3"/>
+      <c r="F199" s="3"/>
     </row>
     <row r="200" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="10"/>
-      <c r="B200" s="10"/>
-      <c r="C200" s="10"/>
-      <c r="D200" s="10"/>
-      <c r="E200" s="10"/>
-      <c r="F200" s="10"/>
+      <c r="A200" s="3"/>
+      <c r="B200" s="3"/>
+      <c r="C200" s="3"/>
+      <c r="D200" s="3"/>
+      <c r="E200" s="3"/>
+      <c r="F200" s="3"/>
     </row>
     <row r="201" spans="1:6" ht="49.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A201" s="10"/>
-      <c r="B201" s="10"/>
-      <c r="C201" s="10"/>
-      <c r="D201" s="10"/>
-      <c r="E201" s="10"/>
-      <c r="F201" s="10"/>
+      <c r="A201" s="4"/>
+      <c r="B201" s="4"/>
+      <c r="C201" s="4"/>
+      <c r="D201" s="4"/>
+      <c r="E201" s="4"/>
+      <c r="F201" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="300">
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="E74:E77"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="D198:D201"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="F198:F201"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D174:D177"/>
+    <mergeCell ref="F174:F177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="D126:D129"/>
+    <mergeCell ref="E94:E97"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="F110:F113"/>
+    <mergeCell ref="D150:D153"/>
+    <mergeCell ref="F150:F153"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="E26:E29"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="A154:A157"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B158:B161"/>
+    <mergeCell ref="E154:E157"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="C98:C101"/>
+    <mergeCell ref="C154:C157"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="B174:B177"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="E198:E201"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="E118:E121"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="D106:D109"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="C138:C141"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="C158:C161"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E194:E197"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="F86:F89"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="D86:D89"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="E162:E165"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="E190:E193"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="F114:F117"/>
     <mergeCell ref="C6:C9"/>
     <mergeCell ref="C62:C65"/>
     <mergeCell ref="A98:A101"/>
@@ -2962,282 +3234,6 @@
     <mergeCell ref="B114:B117"/>
     <mergeCell ref="D114:D117"/>
     <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="F170:F173"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="D86:D89"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="F86:F89"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="C194:C197"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E194:E197"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="E162:E165"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="E134:E137"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="F54:F57"/>
-    <mergeCell ref="C158:C161"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="D106:D109"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="B174:B177"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="E106:E109"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="E198:E201"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="C138:C141"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="C166:C169"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="D170:D173"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="A154:A157"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="E26:E29"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="E74:E77"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="B118:B121"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="E154:E157"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="D198:D201"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="F198:F201"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D174:D177"/>
-    <mergeCell ref="F174:F177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="D126:D129"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="E94:E97"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="F110:F113"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="C98:C101"/>
-    <mergeCell ref="C154:C157"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="D150:D153"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="C118:C121"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>